<commit_message>
Atualização de codigo da vit
</commit_message>
<xml_diff>
--- a/Project_CNN/DenseNet/Resultados/Experimento 2 - DenseNet/training_metrics.xlsx
+++ b/Project_CNN/DenseNet/Resultados/Experimento 2 - DenseNet/training_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci_wawp\Desktop\Arquivos\Mestrado\Projeto-Classificadores\Project_CNN\DenseNet\Resultados\Experimento 2 - DenseNet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF382727-BB10-420D-9D42-EDEFB61C5F51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B807E70F-3580-41F7-8D97-34CBE32C7461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="2520" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -120,7 +120,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="2640" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:defRPr sz="2400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -152,7 +152,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="2640" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="2400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -867,7 +867,7 @@
         <c:axId val="1913391679"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="99"/>
+          <c:max val="100"/>
           <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -879,7 +879,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -911,7 +911,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -948,7 +948,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -998,7 +998,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -1030,7 +1030,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -1062,7 +1062,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -1105,7 +1105,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -1152,7 +1152,7 @@
     <a:lstStyle/>
     <a:p>
       <a:pPr>
-        <a:defRPr sz="2200" baseline="0"/>
+        <a:defRPr sz="2000" baseline="0"/>
       </a:pPr>
       <a:endParaRPr lang="pt-BR"/>
     </a:p>
@@ -1186,7 +1186,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="2640" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:defRPr sz="2400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -1200,11 +1200,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="pt-BR"/>
-              <a:t>DenseNet</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="pt-BR" baseline="0"/>
-              <a:t> - Loss Curves</a:t>
+              <a:t>DenseNet - Loss Curves</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1222,7 +1218,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="2640" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="2400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -1937,7 +1933,7 @@
         <c:axId val="1913393599"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="99"/>
+          <c:max val="100"/>
           <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -1949,7 +1945,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -1981,7 +1977,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -2018,7 +2014,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -2042,6 +2038,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="4.5"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -2066,7 +2063,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -2098,7 +2095,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -2130,7 +2127,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -2172,7 +2169,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="2200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -2219,7 +2216,7 @@
     <a:lstStyle/>
     <a:p>
       <a:pPr>
-        <a:defRPr sz="2200" baseline="0"/>
+        <a:defRPr sz="2000" baseline="0"/>
       </a:pPr>
       <a:endParaRPr lang="pt-BR"/>
     </a:p>
@@ -3350,14 +3347,14 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>2380</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>107156</xdr:rowOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
-      <xdr:colOff>272142</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>9524</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3386,14 +3383,14 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>4481</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>81521</xdr:rowOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
-      <xdr:colOff>272142</xdr:colOff>
-      <xdr:row>58</xdr:row>
-      <xdr:rowOff>59531</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>